<commit_message>
Atualizar planilhas CVM [2026-03-10]
</commit_message>
<xml_diff>
--- a/patrimonio_liquido_cvm_06175696.xlsx
+++ b/patrimonio_liquido_cvm_06175696.xlsx
@@ -438,7 +438,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nome do Fundo/Classe: CV IDEXO FUNDO DE INVESTIMENTO EM PARTICIPAÇÕES MULTIESTRATÉGIA RESPONSABILIDADE LIMITADA CNPJ: 45.615.293/0001-50</t>
+          <t>Nome do Fundo/Classe: ITAÚ SOBERANO RENDA FIXA SIMPLES FIF DA CIC RESPONSABILIDADE LIMITADA CNPJ: 06.175.696/0001-73</t>
         </is>
       </c>
     </row>
@@ -462,7 +462,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>09/2024</t>
+          <t>02/2026</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R$ 82.032.158,38</t>
+          <t>R$ 46.404.535.645,45</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10/10/2024 16:22:16</t>
+          <t>10/03/2026 01:34:03</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,201 +519,41 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ações Descrição: CROMAI TEC AÇÕES CNPJ do emissor: 28.328.465/0001-95 Denominação Social do emissor: CROMAI TECNOLOGIAS AGRÍCOLAS S.A.,</t>
+          <t>Cotas de Fundos</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12000000</v>
+        <v>46409482128</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ações Descrição: DEEP BR AÇÕES CNPJ do emissor: 37.665.648/0001-97 Denominação Social do emissor: DEEP BRASIL INFORMAÇÕES E TECNOLOGIA S.A</t>
+          <t>Disponibilidades</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10000000</v>
+        <v>65693</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ações Descrição: PAYHOP AÇÕES CNPJ do emissor: 35.830.425/0001-02 Denominação Social do emissor: PAYHOP TECNOLOGIA S.A.</t>
+          <t>Valores a pagar</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6500000</v>
+        <v>5060751</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ações Descrição: SMART PROCES ACAO CNPJ do emissor: 28.697.488/0001-77 Denominação Social do emissor: SMART PROCESS S.A.</t>
+          <t>Valores a receber</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>5000000</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Ações Descrição: CARBIG_OP AÇÕES CNPJ do emissor: 30.122.966/0001-62 Denominação Social do emissor: CARBIGDATA TEC E INTEL S.A</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>926072</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Ações Descrição: INTERATALENT AÇÕES CNPJ do emissor: 33.434.173/0001-77 Denominação Social do emissor: INTERA TALENT HACKING RECRUTAMENTO LTDA</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>630000</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Ações Descrição: NFLUX PN CNPJ do emissor: 12.035.640/0001-16 Denominação Social do emissor: NFLUX, INC</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Cotas de Fundos  DAYCOVAL TITULOS PUBLICOS VI FUNDO DE INVESTIMENTO FINANCEIRO CURTO PRAZO</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>1119198.87</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Disponibilidades Descrição: TITULO DE CAIXA CNPJ do emissor: 62.232.889/0001-90 Denominação Social do emissor: BANCO DAYCOVAL S.A.</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>1000</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Investimento no Exterior Nome do emissor: IBBX HOLDINGS LIMITED</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>5347245.28</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Investimento no Exterior Nome do emissor: IBBX HOLDINGS LIMITED</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>3257507.21</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Opções - Posições lançadas Descrição: CARBIGDATA P CNPJ do emissor: 28.697.488/0001-77 Denominação Social do emissor: CARBIGDATA TECNOLOGIA E INT S.A</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Outras aplicações Descrição: INTERA T MÚTUO CNPJ do emissor: 33.434.173/0001-77 Denominação Social do emissor: INTERA TALENT HACKING RECRUTAMENTO LTDA</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>13336191.99</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Outras aplicações Descrição: IBBXHOLD II MÚTUO</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>11004257.88</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Outras aplicações Descrição: CARBIGDATA MUTUO CNPJ do emissor: 30.122.966/0001-62 Denominação Social do emissor: CARBIGDATA TEC E INTEL S.A</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>5687775.15</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Outras aplicações Descrição: INFLEET SOLU MÚTUO CNPJ do emissor: 29.327.781/0001-05 Denominação Social do emissor: INFLEET SOLUÇOES EM TECNOLOGIA LTDA.</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>4050818.16</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Outras aplicações Descrição: INFLEET_SOLU MÚTUO CNPJ do emissor: 29.327.781/0001-05 Denominação Social do emissor: INFLEET SOLUÇOES EM TECNOLOGIA LTDA.</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>3219643.44</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Valores a pagar Descrição: TAXA ADM ADMISTRA CNPJ do emissor: 62.232.889/0001-90 Denominação Social do emissor: BANCO DAYCOVAL S.A.</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>47216.68</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Valores a pagar Descrição: Taxa de Custódia CNPJ do emissor: 62.232.889/0001-90 Denominação Social do emissor: BANCO DAYCOVAL S.A.</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>3500</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Valores a receber Descrição: CVM DIFERIDO CNPJ do emissor: 62.232.889/0001-90 Denominação Social do emissor: BANCO DAYCOVAL S.A.</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>3166.07</v>
+        <v>48575</v>
       </c>
     </row>
   </sheetData>
@@ -727,7 +567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -750,105 +590,53 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Outras aplicações</t>
+          <t>Cotas de Fundos</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>37298686.62</v>
+        <v>46409482128</v>
       </c>
       <c r="C2" t="n">
-        <v>0.4541216269003174</v>
+        <v>0.9998885046380153</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Ações</t>
+          <t>Valores a pagar</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35056073</v>
+        <v>5060751</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4268171977658845</v>
+        <v>0.0001090334672509178</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Investimento no Exterior Nome do emissor: IBBX HOLDINGS LIMITED</t>
+          <t>Disponibilidades</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8604752.49</v>
+        <v>65693</v>
       </c>
       <c r="C4" t="n">
-        <v>0.1047651956124925</v>
+        <v>1.415350323324451e-06</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Cotas de Fundos  DAYCOVAL TITULOS PUBLICOS VI FUNDO DE INVESTIMENTO FINANCEIRO CURTO PRAZO</t>
+          <t>Valores a receber</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1119198.87</v>
+        <v>48575</v>
       </c>
       <c r="C5" t="n">
-        <v>0.01362654982593585</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Valores a pagar</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>50716.68</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.0006174893359444191</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Valores a receber</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>3166.07</v>
-      </c>
-      <c r="C7" t="n">
-        <v>3.854776104929477e-05</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Disponibilidades</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C8" t="n">
-        <v>1.217527125088667e-05</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Opções - Posições lançadas</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>100</v>
-      </c>
-      <c r="C9" t="n">
-        <v>1.217527125088667e-06</v>
+        <v>1.046544410446855e-06</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualizar planilhas CVM [2026-04-30]
</commit_message>
<xml_diff>
--- a/patrimonio_liquido_cvm_06175696.xlsx
+++ b/patrimonio_liquido_cvm_06175696.xlsx
@@ -462,7 +462,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>02/2026</t>
+          <t>03/2026</t>
         </is>
       </c>
     </row>
@@ -474,7 +474,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>R$ 46.404.535.645,45</t>
+          <t>R$ 47.708.047.400,30</t>
         </is>
       </c>
     </row>
@@ -486,7 +486,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10/03/2026 01:34:03</t>
+          <t>09/04/2026 22:20:20</t>
         </is>
       </c>
     </row>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,41 +519,61 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cotas de Fundos</t>
+          <t>Cotas de Fundos  ITAÚ VERSO A RENDA FIXA REFERENCIADO DI FUNDO DE INVESTIMENTO FINANCEIRO RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>46409482128</v>
+        <v>44665680811.11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Disponibilidades</t>
+          <t>Cotas de Fundos  ITAÚ CENTRALIZADOR LFTI11 I FIF RENDA FIXA RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>65693</v>
+        <v>2896955753.89</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Valores a pagar</t>
+          <t>Cotas de Fundos  ITAÚ SOBERANO RENDA FIXA SIMPLES DISTRIBUIDORES FIF CLASSE DE INVESTIMENTO EM COTAS RESP LIMITADA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5060751</v>
+        <v>151536620</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Valores a receber</t>
+          <t>Disponibilidades Descrição: DISPONIBILIDADES</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>48575</v>
+        <v>62287.13</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Valores a pagar Descrição: VALORES A PAGAR</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>6231048.49</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Valores a receber Descrição: VALORES A RECEBER</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>42976.66</v>
       </c>
     </row>
   </sheetData>
@@ -567,7 +587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,53 +610,79 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cotas de Fundos</t>
+          <t>Cotas de Fundos  ITAÚ VERSO A RENDA FIXA REFERENCIADO DI FUNDO DE INVESTIMENTO FINANCEIRO RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>46409482128</v>
+        <v>44665680811.11</v>
       </c>
       <c r="C2" t="n">
-        <v>0.9998885046380153</v>
+        <v>0.9359849943273527</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Valores a pagar</t>
+          <t>Cotas de Fundos  ITAÚ CENTRALIZADOR LFTI11 I FIF RENDA FIXA RESPONSABILIDADE LIMITADA</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5060751</v>
+        <v>2896955753.89</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0001090334672509178</v>
+        <v>0.06070672305070679</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Disponibilidades</t>
+          <t>Cotas de Fundos  ITAÚ SOBERANO RENDA FIXA SIMPLES DISTRIBUIDORES FIF CLASSE DE INVESTIMENTO EM COTAS RESP LIMITADA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>65693</v>
+        <v>151536620</v>
       </c>
       <c r="C4" t="n">
-        <v>1.415350323324451e-06</v>
+        <v>0.003175502977574818</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>Valores a pagar</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>6231048.49</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.0001305738047569496</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Disponibilidades</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>62287.13</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.305248637455354e-06</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>Valores a receber</t>
         </is>
       </c>
-      <c r="B5" t="n">
-        <v>48575</v>
-      </c>
-      <c r="C5" t="n">
-        <v>1.046544410446855e-06</v>
+      <c r="B7" t="n">
+        <v>42976.66</v>
+      </c>
+      <c r="C7" t="n">
+        <v>9.005909713191476e-07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>